<commit_message>
Fix empty summary sheet: inject missing cached formula values (2026-08-31)
The file was built while LibreOffice's recalc engine was unavailable,
leaving every formula cell with an empty <v/> tag instead of a
computed value, which rendered the sheet blank in viewers that don't
recalculate on open.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-08-31.xlsx
+++ b/kirill/outputs/2026-08-31.xlsx
@@ -726,7 +726,7 @@
       </c>
       <c r="C3" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A3,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A3,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>299421.55</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1" s="36">
@@ -740,7 +740,7 @@
       </c>
       <c r="C4" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A4,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A4,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>546513.513</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1" s="36">
@@ -754,7 +754,7 @@
       </c>
       <c r="C5" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A5,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A5,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>82888.624</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1" s="36">
@@ -768,7 +768,7 @@
       </c>
       <c r="C6" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A6,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A6,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>155738.791</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1" s="36">
@@ -782,7 +782,7 @@
       </c>
       <c r="C7" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A7,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A7,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>295436</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1" s="36">
@@ -796,7 +796,7 @@
       </c>
       <c r="C8" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A8,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A8,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>68722.563</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1" s="36">
@@ -810,7 +810,7 @@
       </c>
       <c r="C9" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A9,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A9,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>76847.55</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1" s="36">
@@ -824,7 +824,7 @@
       </c>
       <c r="C10" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A10,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A10,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>4321.85</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="36">
@@ -838,7 +838,7 @@
       </c>
       <c r="C11" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A11,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A11,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>2043.68</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="36">
@@ -852,7 +852,7 @@
       </c>
       <c r="C12" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A12,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A12,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>728.87</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="36">
@@ -866,7 +866,7 @@
       </c>
       <c r="C13" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A13,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A13,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1" s="36">
@@ -880,7 +880,7 @@
       </c>
       <c r="C14" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A14,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A14,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1" s="36">
@@ -894,7 +894,7 @@
       </c>
       <c r="C15" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A15,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A15,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>10118.69</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="36">
@@ -906,7 +906,7 @@
       </c>
       <c r="C16" s="50">
         <f>SUM(C3:C15)</f>
-        <v/>
+        <v>1542781.6810000003</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1" s="36">
@@ -920,7 +920,7 @@
       </c>
       <c r="C17" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A17,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A17,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>391167.74</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="36">
@@ -934,7 +934,7 @@
       </c>
       <c r="C18" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A18,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A18,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>1484.7</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="36">
@@ -946,7 +946,7 @@
       </c>
       <c r="C19" s="50">
         <f>C18+C17+C16</f>
-        <v/>
+        <v>1935434.1210000003</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1" s="36">
@@ -960,7 +960,7 @@
       </c>
       <c r="C20" s="44">
         <f>(Amazon_מקור!B3+Amazon_מקור!B4)*3</f>
-        <v/>
+        <v>202592.25</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1" s="36">
@@ -974,7 +974,7 @@
       </c>
       <c r="C21" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A21,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A21,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>132101.57</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="36">
@@ -988,7 +988,7 @@
       </c>
       <c r="C22" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A22,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A22,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>10986.57</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1" s="36">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="C23" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A23,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A23,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1" s="36">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="C24" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A24,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A24,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="25" ht="14.25" customHeight="1" s="36">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C25" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A25,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A25,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="36">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C26" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A26,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A26,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="36">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C27" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A27,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A27,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="36">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="C28" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A28,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A28,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1" s="36">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="C29" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A29,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A29,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>30237.69</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1" s="36">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="C30" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A30,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A30,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="14.25" customHeight="1" s="36">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C31" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A31,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A31,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" s="36">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="C32" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A32,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A32,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>10037.15</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1" s="36">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="C33" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A33,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A33,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1" s="36">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C34" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A34,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A34,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>18350.05</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1" s="36">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="C35" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A35,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A35,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>26105.72</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1" s="36">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="C36" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A36,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A36,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="14.25" customHeight="1" s="36">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C37" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A37,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A37,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="36">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="C38" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A38,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A38,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="36">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="C39" s="44">
         <f>SUMIF(Pplay1!$F$3:$F$14,A39,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A39,ריכוז!$C$3:$C$30)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="36">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="C40" s="53">
         <f>SUM(C20:C39)</f>
-        <v/>
+        <v>430411</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="36">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="C41" s="55">
         <f>C40+C19</f>
-        <v/>
+        <v>2365845.1210000003</v>
       </c>
     </row>
   </sheetData>
@@ -1336,15 +1336,15 @@
       <c r="E3" s="58" t="n"/>
       <c r="F3" s="61">
         <f>IF(B3&lt;&gt;"",B3,IF(C3&lt;&gt;"",C3,IF(D3&lt;&gt;"",D3,IF(E3&lt;&gt;"",E3,""))))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G3" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A3,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>148904.6</v>
       </c>
       <c r="H3" s="62">
         <f>IF(G3="","",G3*0.91)</f>
-        <v/>
+        <v>135503.186</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1" s="36">
@@ -1361,15 +1361,15 @@
       <c r="E4" s="58" t="n"/>
       <c r="F4" s="61">
         <f>IF(B4&lt;&gt;"",B4,IF(C4&lt;&gt;"",C4,IF(D4&lt;&gt;"",D4,IF(E4&lt;&gt;"",E4,""))))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G4" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A4,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>687.8</v>
       </c>
       <c r="H4" s="62">
         <f>IF(G4="","",G4*0.91)</f>
-        <v/>
+        <v>625.898</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1" s="36">
@@ -1382,17 +1382,17 @@
       <c r="C5" s="58" t="n"/>
       <c r="D5" s="58" t="n"/>
       <c r="E5" s="58" t="n"/>
-      <c r="F5" s="61">
+      <c t="str" r="F5" s="61">
         <f>IF(B5&lt;&gt;"",B5,IF(C5&lt;&gt;"",C5,IF(D5&lt;&gt;"",D5,IF(E5&lt;&gt;"",E5,""))))</f>
         <v/>
       </c>
       <c r="G5" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A5,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>678024.3</v>
       </c>
       <c r="H5" s="62">
         <f>IF(G5="","",G5*0.91)</f>
-        <v/>
+        <v>617002.113</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1" s="36">
@@ -1409,15 +1409,15 @@
       <c r="E6" s="58" t="n"/>
       <c r="F6" s="61">
         <f>IF(B6&lt;&gt;"",B6,IF(C6&lt;&gt;"",C6,IF(D6&lt;&gt;"",D6,IF(E6&lt;&gt;"",E6,""))))</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="G6" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A6,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>3583.7</v>
       </c>
       <c r="H6" s="62">
         <f>IF(G6="","",G6*0.91)</f>
-        <v/>
+        <v>3261.167</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1" s="36">
@@ -1434,15 +1434,15 @@
       <c r="E7" s="58" t="n"/>
       <c r="F7" s="61">
         <f>IF(B7&lt;&gt;"",B7,IF(C7&lt;&gt;"",C7,IF(D7&lt;&gt;"",D7,IF(E7&lt;&gt;"",E7,""))))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G7" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A7,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>58.9</v>
       </c>
       <c r="H7" s="62">
         <f>IF(G7="","",G7*0.91)</f>
-        <v/>
+        <v>53.599</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1" s="36">
@@ -1459,15 +1459,15 @@
       <c r="E8" s="58" t="n"/>
       <c r="F8" s="61">
         <f>IF(B8&lt;&gt;"",B8,IF(C8&lt;&gt;"",C8,IF(D8&lt;&gt;"",D8,IF(E8&lt;&gt;"",E8,""))))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="G8" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A8,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>3566.8</v>
       </c>
       <c r="H8" s="62">
         <f>IF(G8="","",G8*0.91)</f>
-        <v/>
+        <v>3245.788</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1" s="36">
@@ -1484,15 +1484,15 @@
       <c r="E9" s="58" t="n"/>
       <c r="F9" s="61">
         <f>IF(B9&lt;&gt;"",B9,IF(C9&lt;&gt;"",C9,IF(D9&lt;&gt;"",D9,IF(E9&lt;&gt;"",E9,""))))</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="G9" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A9,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>526.9</v>
       </c>
       <c r="H9" s="62">
         <f>IF(G9="","",G9*0.91)</f>
-        <v/>
+        <v>479.479</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1" s="36">
@@ -1509,15 +1509,15 @@
       <c r="E10" s="58" t="n"/>
       <c r="F10" s="61">
         <f>IF(B10&lt;&gt;"",B10,IF(C10&lt;&gt;"",C10,IF(D10&lt;&gt;"",D10,IF(E10&lt;&gt;"",E10,""))))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="G10" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A10,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>600564.3</v>
       </c>
       <c r="H10" s="62">
         <f>IF(G10="","",G10*0.91)</f>
-        <v/>
+        <v>546513.513</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="36">
@@ -1534,15 +1534,15 @@
       <c r="E11" s="58" t="n"/>
       <c r="F11" s="61">
         <f>IF(B11&lt;&gt;"",B11,IF(C11&lt;&gt;"",C11,IF(D11&lt;&gt;"",D11,IF(E11&lt;&gt;"",E11,""))))</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="G11" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A11,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>86975.8</v>
       </c>
       <c r="H11" s="62">
         <f>IF(G11="","",G11*0.91)</f>
-        <v/>
+        <v>79147.978</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="36">
@@ -1559,13 +1559,13 @@
       <c r="E12" s="58" t="n"/>
       <c r="F12" s="61">
         <f>IF(B12&lt;&gt;"",B12,IF(C12&lt;&gt;"",C12,IF(D12&lt;&gt;"",D12,IF(E12&lt;&gt;"",E12,""))))</f>
-        <v/>
-      </c>
-      <c r="G12" s="62">
+        <v>4</v>
+      </c>
+      <c t="str" r="G12" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A12,PPLAY1_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="H12" s="62">
+      <c t="str" r="H12" s="62">
         <f>IF(G12="","",G12*0.91)</f>
         <v/>
       </c>
@@ -1584,15 +1584,15 @@
       </c>
       <c r="F13" s="61">
         <f>IF(B13&lt;&gt;"",B13,IF(C13&lt;&gt;"",C13,IF(D13&lt;&gt;"",D13,IF(E13&lt;&gt;"",E13,""))))</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="G13" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A13,PPLAY1_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>75519.3</v>
       </c>
       <c r="H13" s="62">
         <f>IF(G13="","",G13*0.91)</f>
-        <v/>
+        <v>68722.563</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1" s="36">
@@ -1609,13 +1609,13 @@
       <c r="E14" s="58" t="n"/>
       <c r="F14" s="61">
         <f>IF(B14&lt;&gt;"",B14,IF(C14&lt;&gt;"",C14,IF(D14&lt;&gt;"",D14,IF(E14&lt;&gt;"",E14,""))))</f>
-        <v/>
-      </c>
-      <c r="G14" s="62">
+        <v>4</v>
+      </c>
+      <c t="str" r="G14" s="62">
         <f>IFERROR(INDEX(PPLAY1_מקור!$B:$B,MATCH(A14,PPLAY1_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="H14" s="62">
+      <c t="str" r="H14" s="62">
         <f>IF(G14="","",G14*0.91)</f>
         <v/>
       </c>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="C3" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A3,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>76847.55</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1" s="36">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="C4" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A4,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>299421.55</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1" s="36">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="C5" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A5,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>10118.69</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1" s="36">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C6" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A6,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>2043.68</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1" s="36">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="C7" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A7,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>4321.85</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1" s="36">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="C8" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A8,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>16310.32</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1" s="36">
@@ -1748,7 +1748,7 @@
       <c r="B9" s="35" t="n">
         <v>13</v>
       </c>
-      <c r="C9" s="62">
+      <c t="str" r="C9" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A9,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1762,7 +1762,7 @@
       <c r="B10" s="35" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="62">
+      <c t="str" r="C10" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A10,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="C11" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A11,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>295436</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="36">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="C12" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A12,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>391167.74</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="36">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="C13" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A13,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>1484.7</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1" s="36">
@@ -1818,7 +1818,7 @@
       <c r="B14" s="35" t="n">
         <v>23</v>
       </c>
-      <c r="C14" s="62">
+      <c t="str" r="C14" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A14,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1832,7 +1832,7 @@
       <c r="B15" s="35" t="n">
         <v>25</v>
       </c>
-      <c r="C15" s="62">
+      <c t="str" r="C15" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A15,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="C16" s="62">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A16,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>30237.69</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1" s="36">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="C17" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A17,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>132101.57</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="36">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="C18" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A18,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>26105.72</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1" s="36">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="C19" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A19,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>10986.57</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1" s="36">
@@ -1902,7 +1902,7 @@
       <c r="B20" s="35" t="n">
         <v>22</v>
       </c>
-      <c r="C20" s="64">
+      <c t="str" r="C20" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A20,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1916,7 +1916,7 @@
       <c r="B21" s="35" t="n">
         <v>24</v>
       </c>
-      <c r="C21" s="64">
+      <c t="str" r="C21" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A21,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1930,7 +1930,7 @@
       <c r="B22" s="35" t="n">
         <v>26</v>
       </c>
-      <c r="C22" s="64">
+      <c t="str" r="C22" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A22,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1944,7 +1944,7 @@
       <c r="B23" s="35" t="n">
         <v>27</v>
       </c>
-      <c r="C23" s="64">
+      <c t="str" r="C23" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A23,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1958,7 +1958,7 @@
       <c r="B24" s="35" t="n">
         <v>29</v>
       </c>
-      <c r="C24" s="64">
+      <c t="str" r="C24" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A24,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1972,7 +1972,7 @@
       <c r="B25" s="35" t="n">
         <v>30</v>
       </c>
-      <c r="C25" s="64">
+      <c t="str" r="C25" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A25,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="C26" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A26,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>10037.15</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="36">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="C27" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A27,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>18350.05</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="36">
@@ -2014,7 +2014,7 @@
       <c r="B28" s="35" t="n">
         <v>34</v>
       </c>
-      <c r="C28" s="64">
+      <c t="str" r="C28" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A28,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -2028,7 +2028,7 @@
       <c r="B29" s="35" t="n">
         <v>35</v>
       </c>
-      <c r="C29" s="64">
+      <c t="str" r="C29" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A29,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
       </c>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="C30" s="64">
         <f>IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A30,NetSuite_מקור!$A:$A,0)),"")</f>
-        <v/>
+        <v>728.87</v>
       </c>
     </row>
   </sheetData>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="C2" s="62">
         <f>B2*0.91</f>
-        <v/>
+        <v>135503.186</v>
       </c>
       <c r="D2" s="65" t="n"/>
     </row>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="C3" s="62">
         <f>B3*0.91</f>
-        <v/>
+        <v>625.898</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1" s="36">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="C4" s="62">
         <f>B4*0.91</f>
-        <v/>
+        <v>617002.113</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1" s="36">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="C5" s="62">
         <f>B5*0.91</f>
-        <v/>
+        <v>3261.167</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1" s="36">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="C6" s="62">
         <f>B6*0.91</f>
-        <v/>
+        <v>53.599</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1" s="36">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="C7" s="62">
         <f>B7*0.91</f>
-        <v/>
+        <v>3245.788</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1" s="36">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C8" s="62">
         <f>B8*0.91</f>
-        <v/>
+        <v>479.479</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1" s="36">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="C9" s="62">
         <f>B9*0.91</f>
-        <v/>
+        <v>546513.513</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1" s="36">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="C10" s="62">
         <f>B10*0.91</f>
-        <v/>
+        <v>79147.978</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="36">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="C11" s="35">
         <f>B11*0.91</f>
-        <v/>
+        <v>68722.563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>